<commit_message>
feat: re-run with correct 2010 data pull
</commit_message>
<xml_diff>
--- a/output/five-decade-tables/usa_crowding_by_subgroup_and_decade_raw.xlsx
+++ b/output/five-decade-tables/usa_crowding_by_subgroup_and_decade_raw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ls4540\Documents\dev\households-over-the-years\output\five-decade-tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBF3EC9-D17D-411F-84EE-5469E6B99C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F37CF5C-F2E0-48CB-B6FF-012F06330CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10" yWindow="730" windowWidth="23030" windowHeight="14630" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>row</t>
   </si>
@@ -37,6 +37,9 @@
     <t>2000</t>
   </si>
   <si>
+    <t>2010</t>
+  </si>
+  <si>
     <t>2020</t>
   </si>
   <si>
@@ -49,37 +52,37 @@
     <t>Number of observations</t>
   </si>
   <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>AAPI</t>
+  </si>
+  <si>
+    <t>Hispanic</t>
+  </si>
+  <si>
+    <t>Black</t>
+  </si>
+  <si>
+    <t>AIAN</t>
+  </si>
+  <si>
     <t>White</t>
   </si>
   <si>
-    <t>Hispanic</t>
-  </si>
-  <si>
-    <t>Black</t>
-  </si>
-  <si>
     <t>Multiracial</t>
   </si>
   <si>
-    <t>AIAN</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>AAPI</t>
+    <t>Renter</t>
   </si>
   <si>
     <t>Owner</t>
   </si>
   <si>
-    <t>Renter</t>
+    <t>Foreign-Born</t>
   </si>
   <si>
     <t>U.S.-Born</t>
-  </si>
-  <si>
-    <t>Foreign-Born</t>
   </si>
 </sst>
 </file>
@@ -88,7 +91,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="171" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -140,8 +143,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -447,16 +454,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" customWidth="1"/>
-    <col min="3" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.5703125" customWidth="1"/>
+    <col min="2" max="5" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -475,10 +481,13 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2">
         <v>84.948510276646971</v>
@@ -493,12 +502,15 @@
         <v>89.388300561717102</v>
       </c>
       <c r="F2" s="2">
+        <v>93.797390919725899</v>
+      </c>
+      <c r="G2" s="2">
         <v>94.082423201989059</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2">
         <v>15.051489723353029</v>
@@ -513,12 +525,15 @@
         <v>10.611699438282891</v>
       </c>
       <c r="F3" s="2">
+        <v>6.2026090802741063</v>
+      </c>
+      <c r="G3" s="2">
         <v>5.9175767980109324</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" s="3">
         <v>1972044</v>
@@ -533,242 +548,281 @@
         <v>2740185</v>
       </c>
       <c r="F4" s="3">
+        <v>14757252</v>
+      </c>
+      <c r="G4" s="3">
         <v>14884820</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2">
-        <v>9.1636393508461271</v>
+        <v>29.943502824858761</v>
       </c>
       <c r="C6" s="2">
-        <v>3.4954674809348218</v>
+        <v>14.11992263056093</v>
       </c>
       <c r="D6" s="2">
-        <v>2.7518670442870459</v>
+        <v>25.407685306457701</v>
       </c>
       <c r="E6" s="2">
-        <v>2.4434528470303261</v>
+        <v>16.372483190610659</v>
       </c>
       <c r="F6" s="2">
-        <v>1.474598028368137</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>11.30134029382854</v>
+      </c>
+      <c r="G6" s="2">
+        <v>8.6339384222865814</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2">
-        <v>1.608331254272217</v>
+        <v>23.824583596879609</v>
       </c>
       <c r="C7" s="2">
-        <v>2.0196667841672031</v>
+        <v>25.04198332052486</v>
       </c>
       <c r="D7" s="2">
-        <v>3.3233395970122661</v>
+        <v>28.807203437618181</v>
       </c>
       <c r="E7" s="2">
-        <v>5.0706712198198014</v>
+        <v>25.144343421708282</v>
       </c>
       <c r="F7" s="2">
-        <v>2.8069073238089102</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10.06834273909249</v>
+      </c>
+      <c r="G7" s="2">
+        <v>9.1159877628439574</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2">
-        <v>3.907164343189097</v>
+        <v>41.263790591174022</v>
       </c>
       <c r="C8" s="2">
-        <v>2.3106276745889782</v>
+        <v>30.881477893862861</v>
       </c>
       <c r="D8" s="2">
-        <v>1.911715490446168</v>
+        <v>37.549079127718393</v>
       </c>
       <c r="E8" s="2">
-        <v>1.733242711394672</v>
+        <v>40.192373221292527</v>
       </c>
       <c r="F8" s="2">
-        <v>0.80509496415749704</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19.562518648608481</v>
+      </c>
+      <c r="G8" s="2">
+        <v>14.943219047779831</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
+        <v>13</v>
+      </c>
+      <c r="B9" s="2">
+        <v>35.592664449371767</v>
+      </c>
+      <c r="C9" s="2">
+        <v>20.112411772119991</v>
+      </c>
+      <c r="D9" s="2">
+        <v>16.548801012232179</v>
+      </c>
       <c r="E9" s="2">
-        <v>0.25416249895062792</v>
+        <v>14.778830492261189</v>
       </c>
       <c r="F9" s="2">
-        <v>0.19801009948685011</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>6.9700886242444291</v>
+      </c>
+      <c r="G9" s="2">
+        <v>6.7588238314455653</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" s="2">
-        <v>0.17626381561466181</v>
+        <v>48.097412480974121</v>
       </c>
       <c r="C10" s="2">
-        <v>0.17312851738004881</v>
+        <v>27.10207551179429</v>
       </c>
       <c r="D10" s="2">
-        <v>0.1536459161840725</v>
+        <v>20.323250116256329</v>
       </c>
       <c r="E10" s="2">
-        <v>0.1459524949431221</v>
+        <v>19.868954025441969</v>
       </c>
       <c r="F10" s="2">
-        <v>6.2469916123010803E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>11.70166841734394</v>
+      </c>
+      <c r="G10" s="2">
+        <v>11.47136111949894</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B11" s="2">
-        <v>2.4188101279687471E-2</v>
+        <v>10.91480028097709</v>
       </c>
       <c r="C11" s="2">
-        <v>1.321315396627659E-2</v>
+        <v>4.3885777785605251</v>
       </c>
       <c r="D11" s="2">
-        <v>2.3697239526054709E-2</v>
+        <v>3.624652194244145</v>
       </c>
       <c r="E11" s="2">
-        <v>2.6023002514074231E-2</v>
+        <v>3.5294448630787181</v>
       </c>
       <c r="F11" s="2">
-        <v>3.7223862246941471E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.2389827333642218</v>
+      </c>
+      <c r="G11" s="2">
+        <v>2.5026186360778602</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="2">
-        <v>0.17190285815123801</v>
-      </c>
-      <c r="C12" s="2">
-        <v>0.39811413902500498</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0.8144430697558207</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
       <c r="E12" s="2">
-        <v>0.93819466363026971</v>
+        <v>14.113454968190901</v>
       </c>
       <c r="F12" s="2">
-        <v>0.53327260381958486</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>6.2769406021044336</v>
+      </c>
+      <c r="G12" s="2">
+        <v>5.5673231716507292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B14" s="2">
-        <v>7.3445115829058576</v>
+        <v>23.300504996305278</v>
       </c>
       <c r="C14" s="2">
-        <v>3.8255248269280462</v>
+        <v>15.2006109169906</v>
       </c>
       <c r="D14" s="2">
-        <v>3.3271624938145532</v>
+        <v>17.66511758724921</v>
       </c>
       <c r="E14" s="2">
-        <v>4.1556059616403473</v>
+        <v>20.95878886470399</v>
       </c>
       <c r="F14" s="2">
-        <v>2.2291665102781968</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>12.46149788516572</v>
+      </c>
+      <c r="G14" s="2">
+        <v>11.28582054928777</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B15" s="2">
-        <v>7.7069781404471707</v>
+        <v>10.974478731771329</v>
       </c>
       <c r="C15" s="2">
-        <v>4.5846929231342868</v>
+        <v>5.4776529435395043</v>
       </c>
       <c r="D15" s="2">
-        <v>5.6515458633968736</v>
+        <v>4.8923599106188531</v>
       </c>
       <c r="E15" s="2">
-        <v>6.4560934766425433</v>
+        <v>6.005536600225545</v>
       </c>
       <c r="F15" s="2">
-        <v>3.6884102877327352</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3.1312032349289121</v>
+      </c>
+      <c r="G15" s="2">
+        <v>3.311388005040083</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B17" s="2">
-        <v>14.32158714511441</v>
+        <v>14.143101381492331</v>
       </c>
       <c r="C17" s="2">
-        <v>7.0587655022650146</v>
+        <v>20.149369531044439</v>
       </c>
       <c r="D17" s="2">
-        <v>6.3271414206756598</v>
+        <v>30.390120182644591</v>
       </c>
       <c r="E17" s="2">
-        <v>6.7439871961272164</v>
+        <v>32.582057701254392</v>
       </c>
       <c r="F17" s="2">
-        <v>4.1614928406039908</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15.05452101540356</v>
+      </c>
+      <c r="G17" s="2">
+        <v>11.79177952160955</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B18" s="2">
-        <v>0.72990257823861937</v>
+        <v>15.100921257358561</v>
       </c>
       <c r="C18" s="2">
-        <v>1.351452247797317</v>
+        <v>7.5662464301235497</v>
       </c>
       <c r="D18" s="2">
-        <v>2.6515669365357679</v>
+        <v>6.931961680946551</v>
       </c>
       <c r="E18" s="2">
-        <v>3.867712242155676</v>
+        <v>7.6523764149083533</v>
       </c>
       <c r="F18" s="2">
-        <v>1.7560839574069409</v>
+        <v>4.7819459042574817</v>
+      </c>
+      <c r="G18" s="2">
+        <v>4.8896865935428453</v>
       </c>
     </row>
   </sheetData>

</xml_diff>